<commit_message>
Iterasi 3 - Modifikasi Report Admin Bendahara
</commit_message>
<xml_diff>
--- a/public/assets/templates/Format Import Data Keuangan.xlsx
+++ b/public/assets/templates/Format Import Data Keuangan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Proyek Akhir\sim-almanaar\public\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B32912F8-8324-4D8F-AC67-054237C1E09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A99E9134-1BD1-44A3-AFDB-E2AB5A93929E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{1376679D-98CA-4C2A-A6F0-47AFD37B426B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{1376679D-98CA-4C2A-A6F0-47AFD37B426B}"/>
   </bookViews>
   <sheets>
     <sheet name="DATA IMPORT" sheetId="1" r:id="rId1"/>
@@ -27,9 +27,10 @@
     <definedName name="Kategori_Kas">'DATA MASTER (JANGAN DIUBAH)'!$A$2:$A$5</definedName>
     <definedName name="Komunikasi">'DATA MASTER (JANGAN DIUBAH)'!$G$2</definedName>
     <definedName name="Konsumsi">'DATA MASTER (JANGAN DIUBAH)'!$M$2:$M$3</definedName>
-    <definedName name="Lainnya">'DATA MASTER (JANGAN DIUBAH)'!$P$2</definedName>
+    <definedName name="Lainnya">'DATA MASTER (JANGAN DIUBAH)'!$Q$2:$Q$3</definedName>
     <definedName name="Listrik">'DATA MASTER (JANGAN DIUBAH)'!$L$2</definedName>
     <definedName name="Rawatib">'DATA MASTER (JANGAN DIUBAH)'!$H$2:$H$3</definedName>
+    <definedName name="Santunan">'DATA MASTER (JANGAN DIUBAH)'!$P$2:$P$4</definedName>
     <definedName name="Sholat_Jumat">'DATA MASTER (JANGAN DIUBAH)'!$E$2:$E$6</definedName>
     <definedName name="Taklim">'DATA MASTER (JANGAN DIUBAH)'!$F$2:$F$6</definedName>
     <definedName name="Transportasi">'DATA MASTER (JANGAN DIUBAH)'!$N$2</definedName>
@@ -59,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="66">
   <si>
     <t>Kategori Kas</t>
   </si>
@@ -310,6 +311,21 @@
   </si>
   <si>
     <t>Biaya Taklim Lainnya</t>
+  </si>
+  <si>
+    <t>Dana Lainnya</t>
+  </si>
+  <si>
+    <t>Santunan</t>
+  </si>
+  <si>
+    <t>Yatim</t>
+  </si>
+  <si>
+    <t>Kesejahteraan Umat</t>
+  </si>
+  <si>
+    <t>Bencana</t>
   </si>
 </sst>
 </file>
@@ -395,7 +411,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -430,11 +446,14 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill>
@@ -453,27 +472,6 @@
       <fill>
         <patternFill>
           <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -499,9 +497,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FF1B0B31-C395-49BC-8D28-28F628912C27}" name="Table2" displayName="Table2" ref="A1:P6" totalsRowShown="0" headerRowDxfId="6">
-  <autoFilter ref="A1:P6" xr:uid="{FF1B0B31-C395-49BC-8D28-28F628912C27}"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FF1B0B31-C395-49BC-8D28-28F628912C27}" name="Table2" displayName="Table2" ref="A1:Q6" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:Q6" xr:uid="{FF1B0B31-C395-49BC-8D28-28F628912C27}"/>
+  <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{344F8F2C-DDEA-4C1B-9620-A08FEA1C74BC}" name="Kategori Kas"/>
     <tableColumn id="2" xr3:uid="{9686308A-CB64-4881-ABAB-6B2383183E09}" name="Jenis Transaksi"/>
     <tableColumn id="3" xr3:uid="{8F106D94-9F68-407E-8F66-C9365ECBAB84}" name="Tromol"/>
@@ -517,6 +515,7 @@
     <tableColumn id="13" xr3:uid="{17B52590-66FC-4F9A-8174-B3660C9161F2}" name="Konsumsi"/>
     <tableColumn id="14" xr3:uid="{13D4FC28-864A-4DE5-8027-4E8235919A58}" name="Transportasi"/>
     <tableColumn id="15" xr3:uid="{D989086F-909D-435C-BBE9-8B65EA458A49}" name="Apresiasi"/>
+    <tableColumn id="17" xr3:uid="{B4B3B19F-5A5A-48AE-952B-FCC34CE72380}" name="Santunan"/>
     <tableColumn id="16" xr3:uid="{9A5329E3-2FE3-49B3-BD61-6ACAF6A3914E}" name="Lainnya"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -886,6 +885,7 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
+      <c r="H3" s="12"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
@@ -1888,19 +1888,19 @@
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
+  <conditionalFormatting sqref="A5:G101">
+    <cfRule type="expression" dxfId="2" priority="1">
+      <formula>AND(A5="", COUNTA($A5:$H5)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A5:H101">
-    <cfRule type="expression" dxfId="5" priority="4">
+    <cfRule type="expression" dxfId="1" priority="4">
       <formula>AND(A5&lt;&gt;"", COUNTA($A5:$H5)&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:G101">
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>AND(G5&lt;&gt;"",ISERROR(MATCH(G5,INDIRECT(SUBSTITUTE(F5, " ", "_")),0)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A5:G101">
-    <cfRule type="expression" dxfId="3" priority="1">
-      <formula>AND(A5="", COUNTA($A5:$H5)&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
@@ -1923,7 +1923,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDBBA816-6108-4C9A-9C2E-8CF72BD12C02}">
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.7109375" bestFit="1" customWidth="1"/>
@@ -1940,10 +1940,11 @@
     <col min="13" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="38.140625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.5703125" customWidth="1"/>
+    <col min="17" max="17" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1990,10 +1991,13 @@
         <v>46</v>
       </c>
       <c r="P1" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2040,10 +2044,13 @@
         <v>47</v>
       </c>
       <c r="P2" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2077,8 +2084,14 @@
       <c r="M3" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P3" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2094,8 +2107,11 @@
       <c r="K4" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -2109,7 +2125,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
         <v>16</v>
       </c>

</xml_diff>